<commit_message>
add more datasets for testing + visualization of CV results
</commit_message>
<xml_diff>
--- a/output/reports/cv_experiment_Bagging_kmeans_classification.xlsx
+++ b/output/reports/cv_experiment_Bagging_kmeans_classification.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,23 +491,23 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9002141952514648</v>
+        <v>1.150292873382568</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9983593504958139</v>
+        <v>0.8247979524211558</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9935064935064936</v>
+        <v>0.8435374149659864</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9934996412139632</v>
+        <v>0.8172089314194576</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>0.96343537414966</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>{'max_features': 0.6, 'max_samples': 0.6, 'n_estimators': 25}</t>
+          <t>{'max_features': 0.8, 'max_samples': 0.8, 'n_estimators': 50}</t>
         </is>
       </c>
     </row>
@@ -526,23 +526,58 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>1.457194566726685</v>
+        <v>1.832776308059692</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9983552409841592</v>
+        <v>0.8302894670939711</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9935064935064936</v>
+        <v>0.8367346938775511</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9934996412139632</v>
+        <v>0.7963664405769668</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>0.9614801702994122</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>{'max_features': 0.6, 'max_samples': 0.6, 'n_estimators': 25}</t>
+          <t>{'max_features': 0.8, 'max_samples': 0.8, 'n_estimators': 100}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Bagging</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3.789657831192017</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.8317587282146768</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.8116392379550273</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.9630767272895553</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>{'max_features': 0.8, 'max_samples': 1.0, 'n_estimators': 100}</t>
         </is>
       </c>
     </row>
@@ -557,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -622,23 +657,23 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9002141952514648</v>
+        <v>1.150292873382568</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9983593504958139</v>
+        <v>0.8247979524211558</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9935064935064936</v>
+        <v>0.8435374149659864</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9934996412139632</v>
+        <v>0.8172089314194576</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>0.96343537414966</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>{'max_features': 0.6, 'max_samples': 0.6, 'n_estimators': 25}</t>
+          <t>{'max_features': 0.8, 'max_samples': 0.8, 'n_estimators': 50}</t>
         </is>
       </c>
     </row>
@@ -657,23 +692,58 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>1.457194566726685</v>
+        <v>1.832776308059692</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9983552409841592</v>
+        <v>0.8302894670939711</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9935064935064936</v>
+        <v>0.8367346938775511</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9934996412139632</v>
+        <v>0.7963664405769668</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>0.9614801702994122</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>{'max_features': 0.6, 'max_samples': 0.6, 'n_estimators': 25}</t>
+          <t>{'max_features': 0.8, 'max_samples': 0.8, 'n_estimators': 100}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Bagging</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3.789657831192017</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.8317587282146768</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.8116392379550273</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.9630767272895553</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>{'max_features': 0.8, 'max_samples': 1.0, 'n_estimators': 100}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add scaling for Lasso, Rifge and ElasticNet to avoid non convergence
</commit_message>
<xml_diff>
--- a/output/reports/cv_experiment_Bagging_kmeans_classification.xlsx
+++ b/output/reports/cv_experiment_Bagging_kmeans_classification.xlsx
@@ -491,7 +491,7 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>1.167033195495605</v>
+        <v>1.193494558334351</v>
       </c>
       <c r="E2" t="n">
         <v>0.9983593504958139</v>
@@ -526,7 +526,7 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>1.731572151184082</v>
+        <v>1.790854692459106</v>
       </c>
       <c r="E3" t="n">
         <v>0.9983552409841592</v>
@@ -622,7 +622,7 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>1.167033195495605</v>
+        <v>1.193494558334351</v>
       </c>
       <c r="E2" t="n">
         <v>0.9983593504958139</v>
@@ -657,7 +657,7 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>1.731572151184082</v>
+        <v>1.790854692459106</v>
       </c>
       <c r="E3" t="n">
         <v>0.9983552409841592</v>

</xml_diff>

<commit_message>
add learning curves generation for models expriments
</commit_message>
<xml_diff>
--- a/output/reports/cv_experiment_Bagging_kmeans_classification.xlsx
+++ b/output/reports/cv_experiment_Bagging_kmeans_classification.xlsx
@@ -491,7 +491,7 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7135782241821289</v>
+        <v>0.649118185043335</v>
       </c>
       <c r="E2" t="n">
         <v>0.9983593504958139</v>
@@ -526,7 +526,7 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>1.323484182357788</v>
+        <v>1.075996160507202</v>
       </c>
       <c r="E3" t="n">
         <v>0.9983552409841592</v>
@@ -622,7 +622,7 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7135782241821289</v>
+        <v>0.649118185043335</v>
       </c>
       <c r="E2" t="n">
         <v>0.9983593504958139</v>
@@ -657,7 +657,7 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>1.323484182357788</v>
+        <v>1.075996160507202</v>
       </c>
       <c r="E3" t="n">
         <v>0.9983552409841592</v>

</xml_diff>

<commit_message>
learning curve by CV value
</commit_message>
<xml_diff>
--- a/output/reports/cv_experiment_Bagging_kmeans_classification.xlsx
+++ b/output/reports/cv_experiment_Bagging_kmeans_classification.xlsx
@@ -491,7 +491,7 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.649118185043335</v>
+        <v>0.6855957508087158</v>
       </c>
       <c r="E2" t="n">
         <v>0.9983593504958139</v>
@@ -526,7 +526,7 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>1.075996160507202</v>
+        <v>1.136143445968628</v>
       </c>
       <c r="E3" t="n">
         <v>0.9983552409841592</v>
@@ -622,7 +622,7 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.649118185043335</v>
+        <v>0.6855957508087158</v>
       </c>
       <c r="E2" t="n">
         <v>0.9983593504958139</v>
@@ -657,7 +657,7 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>1.075996160507202</v>
+        <v>1.136143445968628</v>
       </c>
       <c r="E3" t="n">
         <v>0.9983552409841592</v>

</xml_diff>

<commit_message>
add CV value in summary
</commit_message>
<xml_diff>
--- a/output/reports/cv_experiment_Bagging_kmeans_classification.xlsx
+++ b/output/reports/cv_experiment_Bagging_kmeans_classification.xlsx
@@ -491,7 +491,7 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>1.096622705459595</v>
+        <v>0.8900933265686035</v>
       </c>
       <c r="E2" t="n">
         <v>0.9983593504958139</v>
@@ -526,7 +526,7 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>1.609349012374878</v>
+        <v>1.469369411468506</v>
       </c>
       <c r="E3" t="n">
         <v>0.9983552409841592</v>
@@ -561,7 +561,7 @@
         <v>10</v>
       </c>
       <c r="D4" t="n">
-        <v>2.971560955047607</v>
+        <v>2.90601921081543</v>
       </c>
       <c r="E4" t="n">
         <v>0.9983535762483131</v>
@@ -657,7 +657,7 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>1.096622705459595</v>
+        <v>0.8900933265686035</v>
       </c>
       <c r="E2" t="n">
         <v>0.9983593504958139</v>
@@ -692,7 +692,7 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>1.609349012374878</v>
+        <v>1.469369411468506</v>
       </c>
       <c r="E3" t="n">
         <v>0.9983552409841592</v>
@@ -727,7 +727,7 @@
         <v>10</v>
       </c>
       <c r="D4" t="n">
-        <v>2.971560955047607</v>
+        <v>2.90601921081543</v>
       </c>
       <c r="E4" t="n">
         <v>0.9983535762483131</v>

</xml_diff>

<commit_message>
more tests with different datasets
</commit_message>
<xml_diff>
--- a/output/reports/cv_experiment_Bagging_kmeans_classification.xlsx
+++ b/output/reports/cv_experiment_Bagging_kmeans_classification.xlsx
@@ -491,23 +491,23 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>4.598600149154663</v>
+        <v>14.81787252426147</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9280699341723085</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>0.950517836593786</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.932054070173397</v>
+        <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9845430034684587</v>
+        <v>1</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>{'n_estimators': 50, 'max_samples': 0.8, 'max_features': 1.0}</t>
+          <t>{'n_estimators': 100, 'max_samples': 1.0, 'max_features': 0.6}</t>
         </is>
       </c>
     </row>
@@ -526,23 +526,23 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>8.56904125213623</v>
+        <v>27.44591641426086</v>
       </c>
       <c r="E3" t="n">
-        <v>0.928876610929035</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9485040276179517</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9296640638468039</v>
+        <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>0.9831533618758581</v>
+        <v>1</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>{'n_estimators': 25, 'max_samples': 0.6, 'max_features': 1.0}</t>
+          <t>{'n_estimators': 100, 'max_samples': 1.0, 'max_features': 0.6}</t>
         </is>
       </c>
     </row>
@@ -622,23 +622,23 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>4.598600149154663</v>
+        <v>14.81787252426147</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9280699341723085</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>0.950517836593786</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.932054070173397</v>
+        <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9845430034684587</v>
+        <v>1</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>{'n_estimators': 50, 'max_samples': 0.8, 'max_features': 1.0}</t>
+          <t>{'n_estimators': 100, 'max_samples': 1.0, 'max_features': 0.6}</t>
         </is>
       </c>
     </row>
@@ -657,23 +657,23 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>8.56904125213623</v>
+        <v>27.44591641426086</v>
       </c>
       <c r="E3" t="n">
-        <v>0.928876610929035</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9485040276179517</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9296640638468039</v>
+        <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>0.9831533618758581</v>
+        <v>1</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>{'n_estimators': 25, 'max_samples': 0.6, 'max_features': 1.0}</t>
+          <t>{'n_estimators': 100, 'max_samples': 1.0, 'max_features': 0.6}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add more metrics comparaison
</commit_message>
<xml_diff>
--- a/output/reports/cv_experiment_Bagging_kmeans_classification.xlsx
+++ b/output/reports/cv_experiment_Bagging_kmeans_classification.xlsx
@@ -491,7 +491,7 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8552136421203613</v>
+        <v>1.168156385421753</v>
       </c>
       <c r="E2" t="n">
         <v>0.9983593504958139</v>
@@ -526,7 +526,7 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>1.467958688735962</v>
+        <v>2.015239477157593</v>
       </c>
       <c r="E3" t="n">
         <v>0.9983552409841592</v>
@@ -561,7 +561,7 @@
         <v>10</v>
       </c>
       <c r="D4" t="n">
-        <v>2.607017993927002</v>
+        <v>3.985295057296753</v>
       </c>
       <c r="E4" t="n">
         <v>0.9983535762483131</v>
@@ -657,7 +657,7 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8552136421203613</v>
+        <v>1.168156385421753</v>
       </c>
       <c r="E2" t="n">
         <v>0.9983593504958139</v>
@@ -692,7 +692,7 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>1.467958688735962</v>
+        <v>2.015239477157593</v>
       </c>
       <c r="E3" t="n">
         <v>0.9983552409841592</v>
@@ -727,7 +727,7 @@
         <v>10</v>
       </c>
       <c r="D4" t="n">
-        <v>2.607017993927002</v>
+        <v>3.985295057296753</v>
       </c>
       <c r="E4" t="n">
         <v>0.9983535762483131</v>

</xml_diff>

<commit_message>
clean + add new tests
</commit_message>
<xml_diff>
--- a/output/reports/cv_experiment_Bagging_kmeans_classification.xlsx
+++ b/output/reports/cv_experiment_Bagging_kmeans_classification.xlsx
@@ -491,7 +491,7 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>13.85714769363403</v>
+        <v>11.07282543182373</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -526,7 +526,7 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>25.87836480140686</v>
+        <v>21.25451612472534</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -622,7 +622,7 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>13.85714769363403</v>
+        <v>11.07282543182373</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -657,7 +657,7 @@
         <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>25.87836480140686</v>
+        <v>21.25451612472534</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>

</xml_diff>